<commit_message>
chore: use Helene as default for input storm
</commit_message>
<xml_diff>
--- a/data/ARC Storm Surge Shelter Demand.xlsx
+++ b/data/ARC Storm Surge Shelter Demand.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/54fa78dadb255002/Documents/Heinz/Spring 2026/94-739 Capstone/ARC_Capstone/notebooks/repo/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/54fa78dadb255002/Documents/Heinz/Spring 2026/94-739 Capstone/ARC_Capstone/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_9AB5DFE02E429FF0E24E20D6E25A8F1C4D155B9D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_9AB5DFE02E429FF0E24E20D6E25A8F1C4D155B9D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9942B9D2-F76F-441C-A1C5-042FFA90DE54}"/>
   <bookViews>
-    <workbookView xWindow="2240" yWindow="2240" windowWidth="16800" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Interface" sheetId="1" r:id="rId1"/>
@@ -111,13 +111,7 @@
     <t>Storm ID</t>
   </si>
   <si>
-    <t>AL142018</t>
-  </si>
-  <si>
     <t>Storm Name</t>
-  </si>
-  <si>
-    <t>Michael</t>
   </si>
   <si>
     <t>Latest Advisory #</t>
@@ -437,6 +431,12 @@
   </si>
   <si>
     <t>Census tract-level aggregation</t>
+  </si>
+  <si>
+    <t>AL092024</t>
+  </si>
+  <si>
+    <t>Helene</t>
   </si>
 </sst>
 </file>
@@ -1131,6 +1131,26 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1157,27 +1177,7 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1487,40 +1487,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="70.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
     </row>
     <row r="2" spans="1:6" ht="129.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="68"/>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
     </row>
     <row r="3" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="68"/>
+      <c r="B3" s="75"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="76"/>
     </row>
     <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A4" s="70" t="s">
+      <c r="A4" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="71"/>
-      <c r="C4" s="71"/>
-      <c r="D4" s="71"/>
-      <c r="E4" s="71"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
     </row>
     <row r="5" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1"/>
@@ -1530,194 +1530,194 @@
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="62"/>
+      <c r="B6" s="70"/>
       <c r="C6" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="80"/>
+      <c r="E6" s="62"/>
+    </row>
+    <row r="7" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="72"/>
-      <c r="E6" s="73"/>
-    </row>
-    <row r="7" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="61" t="s">
+      <c r="B7" s="70"/>
+      <c r="C7" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="81"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="62"/>
-      <c r="C7" s="5" t="s">
+      <c r="B8" s="70"/>
+      <c r="C8" s="5">
+        <v>16</v>
+      </c>
+      <c r="D8" s="80"/>
+      <c r="E8" s="62"/>
+    </row>
+    <row r="9" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="74"/>
-      <c r="E7" s="73"/>
-      <c r="F7" s="6"/>
-    </row>
-    <row r="8" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="63" t="s">
+      <c r="B9" s="70"/>
+      <c r="C9" s="5">
+        <v>2024</v>
+      </c>
+      <c r="D9" s="80"/>
+      <c r="E9" s="62"/>
+    </row>
+    <row r="10" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="67"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+    </row>
+    <row r="11" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="62"/>
-      <c r="C8" s="5">
-        <v>22</v>
-      </c>
-      <c r="D8" s="72"/>
-      <c r="E8" s="73"/>
-    </row>
-    <row r="9" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="63" t="s">
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="62"/>
+    </row>
+    <row r="12" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="62"/>
-      <c r="C9" s="5">
-        <v>2018</v>
-      </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="73"/>
-    </row>
-    <row r="10" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="75"/>
-      <c r="B10" s="73"/>
-      <c r="C10" s="73"/>
-      <c r="D10" s="73"/>
-      <c r="E10" s="73"/>
-    </row>
-    <row r="11" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="76" t="s">
+      <c r="B12" s="64"/>
+      <c r="C12" s="7" t="s">
         <v>10</v>
-      </c>
-      <c r="B11" s="73"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="73"/>
-    </row>
-    <row r="12" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="77" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="7" t="s">
-        <v>12</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
     <row r="13" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="79" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="78"/>
+      <c r="A13" s="66" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="64"/>
       <c r="C13" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="80" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="78"/>
+      <c r="A14" s="63" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="64"/>
       <c r="C14" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="80" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="78"/>
+      <c r="A15" s="63" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="64"/>
       <c r="C15" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="80" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="78"/>
+      <c r="A16" s="63" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="64"/>
       <c r="C16" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="9"/>
     </row>
     <row r="17" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="79" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="78"/>
+      <c r="A17" s="66" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="64"/>
       <c r="C17" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="9"/>
     </row>
     <row r="18" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="80" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="78"/>
+      <c r="A18" s="63" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="64"/>
       <c r="C18" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="9"/>
     </row>
     <row r="19" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="80" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="78"/>
+      <c r="A19" s="63" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="64"/>
       <c r="C19" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
     </row>
     <row r="20" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="80" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="78"/>
+      <c r="A20" s="63" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="64"/>
       <c r="C20" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
     </row>
     <row r="21" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="80" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="78"/>
+      <c r="A21" s="63" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="64"/>
       <c r="C21" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
     </row>
     <row r="22" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="80" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22" s="78"/>
+      <c r="A22" s="63" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="64"/>
       <c r="C22" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
     </row>
     <row r="23" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="80" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="78"/>
+      <c r="A23" s="63" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="64"/>
       <c r="C23" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
@@ -1730,65 +1730,65 @@
       <c r="E24" s="9"/>
     </row>
     <row r="25" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="81" t="s">
+      <c r="A25" s="61" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="62"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+    </row>
+    <row r="26" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="65" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="64"/>
+      <c r="C26" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="B25" s="73"/>
-      <c r="C25" s="73"/>
-      <c r="D25" s="73"/>
-      <c r="E25" s="73"/>
-    </row>
-    <row r="26" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="77" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="78"/>
-      <c r="C26" s="10" t="s">
-        <v>28</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
     </row>
     <row r="27" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="80" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27" s="78"/>
+      <c r="A27" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="64"/>
       <c r="C27" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
     <row r="28" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="80" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="78"/>
+      <c r="A28" s="63" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="64"/>
       <c r="C28" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
     <row r="29" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="80" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" s="78"/>
+      <c r="A29" s="63" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="64"/>
       <c r="C29" s="11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
     <row r="30" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="80" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30" s="78"/>
+      <c r="A30" s="63" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="64"/>
       <c r="C30" s="12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
@@ -1801,21 +1801,21 @@
       <c r="E31" s="9"/>
     </row>
     <row r="32" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="81" t="s">
+      <c r="A32" s="61" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+    </row>
+    <row r="33" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="65" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="64"/>
+      <c r="C33" s="12" t="s">
         <v>36</v>
-      </c>
-      <c r="B32" s="73"/>
-      <c r="C32" s="73"/>
-      <c r="D32" s="73"/>
-      <c r="E32" s="73"/>
-    </row>
-    <row r="33" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="78"/>
-      <c r="C33" s="12" t="s">
-        <v>38</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
@@ -1828,13 +1828,13 @@
       <c r="E34" s="9"/>
     </row>
     <row r="35" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="81" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35" s="73"/>
-      <c r="C35" s="73"/>
-      <c r="D35" s="73"/>
-      <c r="E35" s="73"/>
+      <c r="A35" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="62"/>
+      <c r="C35" s="62"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="62"/>
     </row>
     <row r="36" spans="1:5" ht="155.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="14"/>
@@ -1851,29 +1851,6 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>
@@ -1886,6 +1863,29 @@
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D9:E9"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C33" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1949,19 +1949,19 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="D1" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="E1" s="22" t="s">
         <v>42</v>
-      </c>
-      <c r="D1" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" s="22" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -1972,13 +1972,13 @@
         <v>4</v>
       </c>
       <c r="C2" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="27" t="s">
         <v>45</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -1986,16 +1986,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -2003,16 +2003,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -2020,16 +2020,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" s="40" t="s">
         <v>52</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="40" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="62.25" customHeight="1" x14ac:dyDescent="0.4">
@@ -2037,10 +2037,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D6" s="44"/>
       <c r="E6" s="45"/>
@@ -2050,16 +2050,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C7" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="46" t="s">
         <v>56</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="46" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2067,16 +2067,16 @@
         <v>2</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C8" s="47" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E8" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2084,16 +2084,16 @@
         <v>2</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2101,16 +2101,16 @@
         <v>2</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C10" s="47" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E10" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2118,16 +2118,16 @@
         <v>2</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C11" s="47" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E11" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2135,16 +2135,16 @@
         <v>2</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C12" s="47" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E12" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2152,16 +2152,16 @@
         <v>2</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C13" s="47" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E13" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2169,16 +2169,16 @@
         <v>2</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C14" s="47" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E14" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2186,16 +2186,16 @@
         <v>2</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C15" s="47" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E15" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2203,16 +2203,16 @@
         <v>2</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C16" s="47" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E16" s="46" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2220,16 +2220,16 @@
         <v>2</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D17" s="49" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2237,10 +2237,10 @@
         <v>3</v>
       </c>
       <c r="B18" s="42" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C18" s="43" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D18" s="52"/>
       <c r="E18" s="53"/>
@@ -2250,16 +2250,16 @@
         <v>3</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C19" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="46" t="s">
         <v>69</v>
-      </c>
-      <c r="D19" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="E19" s="46" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2267,16 +2267,16 @@
         <v>3</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C20" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D20" s="35" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E20" s="46" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2284,16 +2284,16 @@
         <v>3</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C21" s="35" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D21" s="35" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E21" s="46" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2301,16 +2301,16 @@
         <v>3</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C22" s="54" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D22" s="54" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E22" s="51" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2318,10 +2318,10 @@
         <v>3</v>
       </c>
       <c r="B23" s="56" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D23" s="58"/>
       <c r="E23" s="59"/>
@@ -2331,10 +2331,10 @@
         <v>3</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C24" s="35" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D24" s="33"/>
       <c r="E24" s="46"/>
@@ -2344,10 +2344,10 @@
         <v>3</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C25" s="35" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D25" s="33"/>
       <c r="E25" s="46"/>
@@ -2357,10 +2357,10 @@
         <v>3</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D26" s="49"/>
       <c r="E26" s="51"/>
@@ -2370,16 +2370,16 @@
         <v>4</v>
       </c>
       <c r="B27" s="42" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C27" s="43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D27" s="44" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E27" s="59" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.4">
@@ -2387,10 +2387,10 @@
         <v>4</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C28" s="47" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D28" s="60"/>
       <c r="E28" s="46"/>
@@ -2400,10 +2400,10 @@
         <v>4</v>
       </c>
       <c r="B29" s="49" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C29" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D29" s="49"/>
       <c r="E29" s="51"/>

</xml_diff>